<commit_message>
fix(documents): 컨테이너/RORO 계약서(heyman) 상호 SSANCAR→HEYMAN
contract A2:D3 가 SSANCAR 전체 블록(생성 누락분)이라, 컨테이너 인보이스 B3 의
HEYMAN 블록으로 교체(2행 셀이라 한 줄로 평탄화). ⚠ 주소는 아직 싼카(시흥)·이메일
man99777 잔재 — jin 내일 정확한 heyman 주소·연락처로 전 양식 일괄 정리 예정.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/container_contract.xlsx
+++ b/resources/templates/heyman/container_contract.xlsx
@@ -25,7 +25,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Ssancar LTD. Cho Tae Shin. 499, Aam-dero, Yeonsu-gu, Incheon, Korea  Phone: +82-505-366-9977 Email: ssancar9977@gmail.com</t>
+      <t xml:space="preserve">HEYMAN LTD., 163 Sangidaehak-ro, Siheung-si, Gyeonggi-do, Republic of Korea TEL:82-505-355-9977 FAX:82-505-366-9977 EMAIL : man99777@naver.com</t>
     </r>
   </si>
   <si>
@@ -1583,7 +1583,7 @@
       <c r="A2" s="45" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">Ssancar LTD. Cho Tae Shin. 499, Aam-dero, Yeonsu-gu, Incheon, Korea  Phone: +82-505-366-9977 Email: ssancar9977@gmail.com</t>
+            <t xml:space="preserve">HEYMAN LTD., 163 Sangidaehak-ro, Siheung-si, Gyeonggi-do, Republic of Korea TEL:82-505-355-9977 FAX:82-505-366-9977 EMAIL : man99777@naver.com</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
fix(templates): 서류에 잘못 박힌 전화번호 정정 (heyman 3건 · karaba 1건)
판매계약서 정본을 맞추려고 3사 × 5서류 연락처를 전수 대조하다 나온 교차오염.
jin 2026-07-29 확인: heyman Tel 82-10-9009-9977 / Fax 82-505-366-9977, karaba Tel 82-32-710-7979.

- heyman roro/container 계약서 A2 : TEL 이 ssancar 대표번호(82-505-355-9977) 였음
- heyman 인보이스 A2             : Phone 자리에 팩스번호(82-505-366-9977) 가 있었음
- karaba 말소계약서 E4           : heyman 번호(82-10-9009-9977) 가 박혀 있었음

대상 셀이 전부 RichText 라 setValue 로 덮으면 헤더 서식이 날아간다 → run 텍스트만
부분치환(scripts/fix-template-phone-numbers.php, --dry 지원). 4개 파일 재로드 검증
(definedNames 0 유지) + 서류 생성 테스트 113 통과.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/container_contract.xlsx
+++ b/resources/templates/heyman/container_contract.xlsx
@@ -25,7 +25,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">HEYMAN LTD., #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea TEL:82-505-355-9977 FAX:82-505-366-9977 EMAIL : heyman99888@gmail.com</t>
+      <t xml:space="preserve">HEYMAN LTD., #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea TEL:82-10-9009-9977 FAX:82-505-366-9977 EMAIL : heyman99888@gmail.com</t>
     </r>
   </si>
   <si>
@@ -1570,7 +1570,7 @@
       <c r="A2" s="45" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">HEYMAN LTD., #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea TEL:82-505-355-9977 FAX:82-505-366-9977 EMAIL : heyman99888@gmail.com</t>
+            <t xml:space="preserve">HEYMAN LTD., #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea TEL:82-10-9009-9977 FAX:82-505-366-9977 EMAIL : heyman99888@gmail.com</t>
           </r>
         </is>
       </c>

</xml_diff>